<commit_message>
Follow observed website category and default product order instead of price or bestseller ranking
</commit_message>
<xml_diff>
--- a/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
+++ b/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
@@ -1893,7 +1893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG1"/>
+  <dimension ref="A1:AM1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2094,6 +2094,36 @@
       <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>analysis_note</t>
+        </is>
+      </c>
+      <c r="AH1" s="4" t="inlineStr">
+        <is>
+          <t>website_category_order</t>
+        </is>
+      </c>
+      <c r="AI1" s="4" t="inlineStr">
+        <is>
+          <t>website_subcategory_order</t>
+        </is>
+      </c>
+      <c r="AJ1" s="4" t="inlineStr">
+        <is>
+          <t>website_product_order</t>
+        </is>
+      </c>
+      <c r="AK1" s="4" t="inlineStr">
+        <is>
+          <t>website_order_source_url</t>
+        </is>
+      </c>
+      <c r="AL1" s="4" t="inlineStr">
+        <is>
+          <t>website_order_checked_at</t>
+        </is>
+      </c>
+      <c r="AM1" s="4" t="inlineStr">
+        <is>
+          <t>website_order_status</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Require exact source category evidence and validate before fresh restart
</commit_message>
<xml_diff>
--- a/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
+++ b/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
@@ -1893,7 +1893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM1"/>
+  <dimension ref="A1:AQ1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2124,6 +2124,26 @@
       <c r="AM1" s="4" t="inlineStr">
         <is>
           <t>website_order_status</t>
+        </is>
+      </c>
+      <c r="AN1" s="4" t="inlineStr">
+        <is>
+          <t>website_category_path</t>
+        </is>
+      </c>
+      <c r="AO1" s="4" t="inlineStr">
+        <is>
+          <t>website_category_source_url</t>
+        </is>
+      </c>
+      <c r="AP1" s="4" t="inlineStr">
+        <is>
+          <t>website_category_checked_at</t>
+        </is>
+      </c>
+      <c r="AQ1" s="4" t="inlineStr">
+        <is>
+          <t>website_category_status</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Infer missing subcategories from product text with explicit provenance
</commit_message>
<xml_diff>
--- a/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
+++ b/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
@@ -326,6 +326,21 @@
         <t>Internal Rule 804 research note: record observed bestseller-sort position, product-page merchant labels, named collection membership, source URLs, check times and uncertainty. Top/featured collection names alone do not prove sales. Preserve as plain text; do not display automatically as customer product description.</t>
       </text>
     </comment>
+    <comment ref="AR1" authorId="0" shapeId="0">
+      <text>
+        <t>website, inferred_description, inferred_product_name, existing, or unverified. Inferred labels are not verified website taxonomy.</t>
+      </text>
+    </comment>
+    <comment ref="AS1" authorId="0" shapeId="0">
+      <text>
+        <t>Exact observed website path or short quote from supplied name/description supporting the inferred product type.</t>
+      </text>
+    </comment>
+    <comment ref="AT1" authorId="0" shapeId="0">
+      <text>
+        <t>ISO-8601 check time; blank when the type remains unverified.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -573,13 +588,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="B2:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -594,7 +608,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -616,7 +629,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -652,7 +664,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
@@ -681,7 +692,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
@@ -703,7 +713,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
@@ -718,7 +727,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
@@ -733,7 +741,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -762,7 +769,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="B35" s="2" t="inlineStr">
         <is>
@@ -770,7 +776,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="B37" s="3" t="inlineStr">
         <is>
@@ -1893,7 +1898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ1"/>
+  <dimension ref="A1:AT1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1928,6 +1933,9 @@
     <col width="55" customWidth="1" min="31" max="31"/>
     <col width="25" customWidth="1" min="32" max="32"/>
     <col width="80" customWidth="1" min="33" max="33"/>
+    <col width="38" customWidth="1" min="44" max="44"/>
+    <col width="38" customWidth="1" min="45" max="45"/>
+    <col width="38" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2144,6 +2152,21 @@
       <c r="AQ1" s="4" t="inlineStr">
         <is>
           <t>website_category_status</t>
+        </is>
+      </c>
+      <c r="AR1" s="4" t="inlineStr">
+        <is>
+          <t>subcategory_source</t>
+        </is>
+      </c>
+      <c r="AS1" s="4" t="inlineStr">
+        <is>
+          <t>subcategory_evidence</t>
+        </is>
+      </c>
+      <c r="AT1" s="4" t="inlineStr">
+        <is>
+          <t>subcategory_checked_at</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lock shop-coded Category-only template and retain all existing classification values
</commit_message>
<xml_diff>
--- a/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
+++ b/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
@@ -942,7 +942,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>• category: groups products into tabs in the app, in the order they first appear. subcategory/sku/source_url are kept for reference only.</t>
+          <t>• Category: the single final category label, renamed from the former subcategory column. shop_code is first; confirmed codes repeat on every product and unknown stores stay blank. sku/source_url and subcategory_* evidence fields remain reference/audit data.</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
     <row r="3">
       <c r="A3" s="30" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B3" s="30" t="inlineStr">
@@ -1082,19 +1082,19 @@
       </c>
       <c r="C3" s="30" t="inlineStr">
         <is>
-          <t>Tab/section in the shop</t>
+          <t>Final product category label, formerly exported as subcategory; website evidence first, labelled text inference when missing.</t>
         </is>
       </c>
       <c r="D3" s="30" t="inlineStr">
         <is>
-          <t>Shirts</t>
+          <t>Face Wash</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="30" t="inlineStr">
         <is>
-          <t>subcategory</t>
+          <t>subcategory_source</t>
         </is>
       </c>
       <c r="B4" s="30" t="inlineStr">
@@ -1104,12 +1104,12 @@
       </c>
       <c r="C4" s="30" t="inlineStr">
         <is>
-          <t>Reference only</t>
+          <t>Audit provenance only: website, inferred_description, inferred_product_name, existing or unverified.</t>
         </is>
       </c>
       <c r="D4" s="30" t="inlineStr">
         <is>
-          <t>Men</t>
+          <t>website</t>
         </is>
       </c>
     </row>
@@ -1901,8 +1901,8 @@
   <dimension ref="A1:AT1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
@@ -1941,17 +1941,17 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
+          <t>shop_code</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
           <t>product_id</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>subcategory</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
@@ -2171,9 +2171,9 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:A5000">
+  <conditionalFormatting sqref="B2:B5000">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND($A2&lt;&gt;"",COUNTIF($A$2:$A$5000,$A2)&gt;1)</formula>
+      <formula>AND($B2&lt;&gt;"",COUNTIF($B$2:$B$5000,$B2)&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="7">

</xml_diff>

<commit_message>
Classify catalog products by intended purpose and preserve source taxonomy
</commit_message>
<xml_diff>
--- a/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
+++ b/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
@@ -328,7 +328,7 @@
     </comment>
     <comment ref="AR1" authorId="0" shapeId="0">
       <text>
-        <t>website, inferred_description, inferred_product_name, existing, or unverified. Inferred labels are not verified website taxonomy.</t>
+        <t>website, inferred_description, inferred_product_name, inferred_product_type, manual, existing, or unverified. Public product types are distinct from factual website taxonomy.</t>
       </text>
     </comment>
     <comment ref="AS1" authorId="0" shapeId="0">
@@ -723,7 +723,7 @@
     <row r="25">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Products mein nayi row: product_id (unique), category, subcategory, name, description, brand, material, base_price (aur agar discount ho to sale_price), option_groups.</t>
+          <t>Products: shop_code, product_id (unique), Category, name, description, brand, material, base_price, sale_price and option_groups. Category is the supported product type; website path and inference evidence remain separate.</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="C3" s="30" t="inlineStr">
         <is>
-          <t>Final product category label, formerly exported as subcategory; website evidence first, labelled text inference when missing.</t>
+          <t>Consistent product type from explicit product name and descriptive purpose. Refine broad collection labels; retain original website taxonomy separately. Ignore ingredient and application-tool mentions. Unclear types require review.</t>
         </is>
       </c>
       <c r="D3" s="30" t="inlineStr">

</xml_diff>

<commit_message>
Label variant image provenance and same-product fallback without inventing image or stock mappings
</commit_message>
<xml_diff>
--- a/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
+++ b/importer-files/Chotu_Products_Import_Template_Discount_Tags.xlsx
@@ -2582,7 +2582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -2708,6 +2708,21 @@
           <t>source_discount_tag</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>variant_image_status</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>fallback_image_url</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>variant_image_note</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>